<commit_message>
screener: relatório de 2026-08-04
</commit_message>
<xml_diff>
--- a/reports/screener_2026-08-04.xlsx
+++ b/reports/screener_2026-08-04.xlsx
@@ -1371,7 +1371,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW5" t="n">
@@ -1725,10 +1725,10 @@
         </is>
       </c>
       <c r="AW7" t="n">
-        <v>5.639999866485596</v>
+        <v>5.619999885559082</v>
       </c>
       <c r="AX7" t="n">
-        <v>-14.71631105238386</v>
+        <v>-14.41281066323299</v>
       </c>
       <c r="AY7" t="n">
         <v>-39.50409545018086</v>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>sem sinal (-14.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -2240,10 +2240,10 @@
         </is>
       </c>
       <c r="AW10" t="n">
-        <v>19.21999931335449</v>
+        <v>18.85000038146973</v>
       </c>
       <c r="AX10" t="n">
-        <v>-16.54525760371704</v>
+        <v>-14.90715866883865</v>
       </c>
       <c r="AY10" t="n">
         <v>-54.13720844041888</v>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="BC10" t="inlineStr">
         <is>
-          <t>sem sinal (-16.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW13" t="n">
@@ -2773,7 +2773,7 @@
         <v>-3.612203515041446</v>
       </c>
       <c r="AY13" t="n">
-        <v>-22.7763666994001</v>
+        <v>-22.77636138240788</v>
       </c>
       <c r="AZ13" t="b">
         <v>1</v>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.6% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -2944,10 +2944,10 @@
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>13</v>
+        <v>12.72999954223633</v>
       </c>
       <c r="AX14" t="n">
-        <v>-14.30768966674805</v>
+        <v>-12.4901748318072</v>
       </c>
       <c r="AY14" t="n">
         <v>-32.85678377733036</v>
@@ -2963,7 +2963,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>sem sinal (-14.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-12.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -3282,10 +3282,10 @@
         </is>
       </c>
       <c r="AW16" t="n">
-        <v>43.04999923706055</v>
+        <v>43.41999816894531</v>
       </c>
       <c r="AX16" t="n">
-        <v>-1.277582454837922</v>
+        <v>-2.118835116863982</v>
       </c>
       <c r="AY16" t="n">
         <v>-13.54395936495905</v>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="BC16" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-2.1% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -4336,10 +4336,10 @@
         </is>
       </c>
       <c r="AW22" t="n">
-        <v>48.70000076293945</v>
+        <v>49.04000091552734</v>
       </c>
       <c r="AX22" t="n">
-        <v>-1.129361865388501</v>
+        <v>-1.814843745989081</v>
       </c>
       <c r="AY22" t="n">
         <v>-11.83384458058885</v>
@@ -4355,7 +4355,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-1.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -4859,10 +4859,10 @@
         </is>
       </c>
       <c r="AW25" t="n">
-        <v>6.579999923706055</v>
+        <v>6.550000190734863</v>
       </c>
       <c r="AX25" t="n">
-        <v>-3.49544105988292</v>
+        <v>-3.053439393562163</v>
       </c>
       <c r="AY25" t="n">
         <v>-39.52381043207078</v>
@@ -4878,7 +4878,7 @@
       </c>
       <c r="BC25" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.1% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
         <v>-2.713682693188602</v>
       </c>
       <c r="AY27" t="n">
-        <v>-39.5192605242667</v>
+        <v>-39.51925229062647</v>
       </c>
       <c r="AZ27" t="b">
         <v>1</v>
@@ -6557,7 +6557,7 @@
       <c r="AU35" t="inlineStr"/>
       <c r="AV35" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW35" t="n">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="BC35" t="inlineStr">
         <is>
-          <t>sem sinal (-2.2% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
         <v>-3.347322770539629</v>
       </c>
       <c r="AY36" t="n">
-        <v>-12.30894652743484</v>
+        <v>-12.30895602838301</v>
       </c>
       <c r="AZ36" t="b">
         <v>1</v>
@@ -7076,10 +7076,10 @@
         </is>
       </c>
       <c r="AW38" t="n">
-        <v>29.75</v>
+        <v>29.73999977111816</v>
       </c>
       <c r="AX38" t="n">
-        <v>-2.285715311515235</v>
+        <v>-2.252858377438904</v>
       </c>
       <c r="AY38" t="n">
         <v>-17.59775069846685</v>
@@ -7249,10 +7249,10 @@
         </is>
       </c>
       <c r="AW39" t="n">
-        <v>3.980000019073486</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="AX39" t="n">
-        <v>-0.7537681217588132</v>
+        <v>-1.98511558212644</v>
       </c>
       <c r="AY39" t="n">
         <v>-47.92224740248528</v>
@@ -7268,7 +7268,7 @@
       </c>
       <c r="BC39" t="inlineStr">
         <is>
-          <t>sem sinal (-0.8% do topo; Lateral)</t>
+          <t>sem sinal (-2.0% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -7603,10 +7603,10 @@
         </is>
       </c>
       <c r="AW41" t="n">
-        <v>2.339999914169312</v>
+        <v>2.329999923706055</v>
       </c>
       <c r="AX41" t="n">
-        <v>-3.418800283779255</v>
+        <v>-3.004289078750577</v>
       </c>
       <c r="AY41" t="n">
         <v>-52.18694930098489</v>
@@ -7622,7 +7622,7 @@
       </c>
       <c r="BC41" t="inlineStr">
         <is>
-          <t>sem sinal (-3.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -8639,7 +8639,7 @@
         <v>-3.855259824575719</v>
       </c>
       <c r="AY47" t="n">
-        <v>-14.20840116822351</v>
+        <v>-14.20839330687329</v>
       </c>
       <c r="AZ47" t="b">
         <v>1</v>
@@ -8975,10 +8975,10 @@
         </is>
       </c>
       <c r="AW49" t="n">
-        <v>11.27999973297119</v>
+        <v>11.34000015258789</v>
       </c>
       <c r="AX49" t="n">
-        <v>0</v>
+        <v>-0.5291042223046771</v>
       </c>
       <c r="AY49" t="n">
         <v>-15.4147281673955</v>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="BC49" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Alta)</t>
+          <t>sem sinal (-0.5% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -9152,10 +9152,10 @@
         </is>
       </c>
       <c r="AW50" t="n">
-        <v>16.3700008392334</v>
+        <v>16.1200008392334</v>
       </c>
       <c r="AX50" t="n">
-        <v>-14.84423417392992</v>
+        <v>-13.52358030617676</v>
       </c>
       <c r="AY50" t="n">
         <v>-34.85117715011583</v>
@@ -9171,7 +9171,7 @@
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>sem sinal (-14.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-13.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -9321,14 +9321,14 @@
       <c r="AU51" t="inlineStr"/>
       <c r="AV51" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW51" t="n">
-        <v>43.09999847412109</v>
+        <v>43.31999969482422</v>
       </c>
       <c r="AX51" t="n">
-        <v>-0.1856102533401627</v>
+        <v>-0.6925190193304398</v>
       </c>
       <c r="AY51" t="n">
         <v>-27.87197279000151</v>
@@ -9344,7 +9344,7 @@
       </c>
       <c r="BC51" t="inlineStr">
         <is>
-          <t>sem sinal (-0.2% do topo; Lateral)</t>
+          <t>sem sinal (-0.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -9862,7 +9862,7 @@
         <v>-4.576970169490013</v>
       </c>
       <c r="AY54" t="n">
-        <v>-23.4739172343906</v>
+        <v>-23.47392377028176</v>
       </c>
       <c r="AZ54" t="b">
         <v>1</v>
@@ -10846,7 +10846,7 @@
       <c r="AU60" t="inlineStr"/>
       <c r="AV60" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW60" t="n">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="BC60" t="inlineStr">
         <is>
-          <t>sem sinal (-2.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.7% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -11498,13 +11498,13 @@
         </is>
       </c>
       <c r="AW64" t="n">
-        <v>43.63000106811523</v>
+        <v>43.61150741577148</v>
       </c>
       <c r="AX64" t="n">
-        <v>-3.506767262291599</v>
+        <v>-3.465848880756128</v>
       </c>
       <c r="AY64" t="n">
-        <v>-13.58725425550743</v>
+        <v>-13.55060269313266</v>
       </c>
       <c r="AZ64" t="b">
         <v>1</v>
@@ -11852,10 +11852,10 @@
         </is>
       </c>
       <c r="AW66" t="n">
-        <v>76.08999633789062</v>
+        <v>76.27999877929688</v>
       </c>
       <c r="AX66" t="n">
-        <v>0.2891329100952689</v>
+        <v>0.03932718901014098</v>
       </c>
       <c r="AY66" t="n">
         <v>-16.71033041805866</v>
@@ -13002,7 +13002,7 @@
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW5" t="n">
@@ -13356,10 +13356,10 @@
         </is>
       </c>
       <c r="AW7" t="n">
-        <v>5.639999866485596</v>
+        <v>5.619999885559082</v>
       </c>
       <c r="AX7" t="n">
-        <v>-14.71631105238386</v>
+        <v>-14.41281066323299</v>
       </c>
       <c r="AY7" t="n">
         <v>-39.50409545018086</v>
@@ -13375,7 +13375,7 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>sem sinal (-14.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -13871,10 +13871,10 @@
         </is>
       </c>
       <c r="AW10" t="n">
-        <v>19.21999931335449</v>
+        <v>18.85000038146973</v>
       </c>
       <c r="AX10" t="n">
-        <v>-16.54525760371704</v>
+        <v>-14.90715866883865</v>
       </c>
       <c r="AY10" t="n">
         <v>-54.13720844041888</v>
@@ -13890,7 +13890,7 @@
       </c>
       <c r="BC10" t="inlineStr">
         <is>
-          <t>sem sinal (-16.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -14394,7 +14394,7 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW13" t="n">
@@ -14404,7 +14404,7 @@
         <v>-3.612203515041446</v>
       </c>
       <c r="AY13" t="n">
-        <v>-22.7763666994001</v>
+        <v>-22.77636138240788</v>
       </c>
       <c r="AZ13" t="b">
         <v>1</v>
@@ -14417,7 +14417,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.6% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -14575,10 +14575,10 @@
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>13</v>
+        <v>12.72999954223633</v>
       </c>
       <c r="AX14" t="n">
-        <v>-14.30768966674805</v>
+        <v>-12.4901748318072</v>
       </c>
       <c r="AY14" t="n">
         <v>-32.85678377733036</v>
@@ -14594,7 +14594,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>sem sinal (-14.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-12.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -14913,10 +14913,10 @@
         </is>
       </c>
       <c r="AW16" t="n">
-        <v>43.04999923706055</v>
+        <v>43.41999816894531</v>
       </c>
       <c r="AX16" t="n">
-        <v>-1.277582454837922</v>
+        <v>-2.118835116863982</v>
       </c>
       <c r="AY16" t="n">
         <v>-13.54395936495905</v>
@@ -14932,7 +14932,7 @@
       </c>
       <c r="BC16" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-2.1% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -15967,10 +15967,10 @@
         </is>
       </c>
       <c r="AW22" t="n">
-        <v>48.70000076293945</v>
+        <v>49.04000091552734</v>
       </c>
       <c r="AX22" t="n">
-        <v>-1.129361865388501</v>
+        <v>-1.814843745989081</v>
       </c>
       <c r="AY22" t="n">
         <v>-11.83384458058885</v>
@@ -15986,7 +15986,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-1.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -16657,10 +16657,10 @@
         </is>
       </c>
       <c r="AW26" t="n">
-        <v>6.579999923706055</v>
+        <v>6.550000190734863</v>
       </c>
       <c r="AX26" t="n">
-        <v>-3.49544105988292</v>
+        <v>-3.053439393562163</v>
       </c>
       <c r="AY26" t="n">
         <v>-39.52381043207078</v>
@@ -16676,7 +16676,7 @@
       </c>
       <c r="BC26" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.1% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -17021,7 +17021,7 @@
         <v>-2.713682693188602</v>
       </c>
       <c r="AY28" t="n">
-        <v>-39.5192605242667</v>
+        <v>-39.51925229062647</v>
       </c>
       <c r="AZ28" t="b">
         <v>1</v>
@@ -18355,7 +18355,7 @@
       <c r="AU36" t="inlineStr"/>
       <c r="AV36" t="inlineStr">
         <is>
-          <t>Em Alta</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW36" t="n">
@@ -18378,7 +18378,7 @@
       </c>
       <c r="BC36" t="inlineStr">
         <is>
-          <t>sem sinal (-2.2% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -18530,7 +18530,7 @@
         <v>-3.347322770539629</v>
       </c>
       <c r="AY37" t="n">
-        <v>-12.30894652743484</v>
+        <v>-12.30895602838301</v>
       </c>
       <c r="AZ37" t="b">
         <v>1</v>
@@ -18874,10 +18874,10 @@
         </is>
       </c>
       <c r="AW39" t="n">
-        <v>29.75</v>
+        <v>29.73999977111816</v>
       </c>
       <c r="AX39" t="n">
-        <v>-2.285715311515235</v>
+        <v>-2.252858377438904</v>
       </c>
       <c r="AY39" t="n">
         <v>-17.59775069846685</v>
@@ -19047,10 +19047,10 @@
         </is>
       </c>
       <c r="AW40" t="n">
-        <v>3.980000019073486</v>
+        <v>4.03000020980835</v>
       </c>
       <c r="AX40" t="n">
-        <v>-0.7537681217588132</v>
+        <v>-1.98511558212644</v>
       </c>
       <c r="AY40" t="n">
         <v>-47.92224740248528</v>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="BC40" t="inlineStr">
         <is>
-          <t>sem sinal (-0.8% do topo; Lateral)</t>
+          <t>sem sinal (-2.0% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -19401,10 +19401,10 @@
         </is>
       </c>
       <c r="AW42" t="n">
-        <v>2.339999914169312</v>
+        <v>2.329999923706055</v>
       </c>
       <c r="AX42" t="n">
-        <v>-3.418800283779255</v>
+        <v>-3.004289078750577</v>
       </c>
       <c r="AY42" t="n">
         <v>-52.18694930098489</v>
@@ -19420,7 +19420,7 @@
       </c>
       <c r="BC42" t="inlineStr">
         <is>
-          <t>sem sinal (-3.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-3.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -20437,7 +20437,7 @@
         <v>-3.855259824575719</v>
       </c>
       <c r="AY48" t="n">
-        <v>-14.20840116822351</v>
+        <v>-14.20839330687329</v>
       </c>
       <c r="AZ48" t="b">
         <v>1</v>
@@ -20773,10 +20773,10 @@
         </is>
       </c>
       <c r="AW50" t="n">
-        <v>11.27999973297119</v>
+        <v>11.34000015258789</v>
       </c>
       <c r="AX50" t="n">
-        <v>0</v>
+        <v>-0.5291042223046771</v>
       </c>
       <c r="AY50" t="n">
         <v>-15.4147281673955</v>
@@ -20792,7 +20792,7 @@
       </c>
       <c r="BC50" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Alta)</t>
+          <t>sem sinal (-0.5% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -20950,10 +20950,10 @@
         </is>
       </c>
       <c r="AW51" t="n">
-        <v>16.3700008392334</v>
+        <v>16.1200008392334</v>
       </c>
       <c r="AX51" t="n">
-        <v>-14.84423417392992</v>
+        <v>-13.52358030617676</v>
       </c>
       <c r="AY51" t="n">
         <v>-34.85117715011583</v>
@@ -20969,7 +20969,7 @@
       </c>
       <c r="BC51" t="inlineStr">
         <is>
-          <t>sem sinal (-14.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-13.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -21119,14 +21119,14 @@
       <c r="AU52" t="inlineStr"/>
       <c r="AV52" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW52" t="n">
-        <v>43.09999847412109</v>
+        <v>43.31999969482422</v>
       </c>
       <c r="AX52" t="n">
-        <v>-0.1856102533401627</v>
+        <v>-0.6925190193304398</v>
       </c>
       <c r="AY52" t="n">
         <v>-27.87197279000151</v>
@@ -21142,7 +21142,7 @@
       </c>
       <c r="BC52" t="inlineStr">
         <is>
-          <t>sem sinal (-0.2% do topo; Lateral)</t>
+          <t>sem sinal (-0.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -21660,7 +21660,7 @@
         <v>-4.576970169490013</v>
       </c>
       <c r="AY55" t="n">
-        <v>-23.4739172343906</v>
+        <v>-23.47392377028176</v>
       </c>
       <c r="AZ55" t="b">
         <v>1</v>
@@ -22644,7 +22644,7 @@
       <c r="AU61" t="inlineStr"/>
       <c r="AV61" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW61" t="n">
@@ -22667,7 +22667,7 @@
       </c>
       <c r="BC61" t="inlineStr">
         <is>
-          <t>sem sinal (-2.7% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.7% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -23296,13 +23296,13 @@
         </is>
       </c>
       <c r="AW65" t="n">
-        <v>43.63000106811523</v>
+        <v>43.61150741577148</v>
       </c>
       <c r="AX65" t="n">
-        <v>-3.506767262291599</v>
+        <v>-3.465848880756128</v>
       </c>
       <c r="AY65" t="n">
-        <v>-13.58725425550743</v>
+        <v>-13.55060269313266</v>
       </c>
       <c r="AZ65" t="b">
         <v>1</v>
@@ -23650,10 +23650,10 @@
         </is>
       </c>
       <c r="AW67" t="n">
-        <v>76.08999633789062</v>
+        <v>76.27999877929688</v>
       </c>
       <c r="AX67" t="n">
-        <v>0.2891329100952689</v>
+        <v>0.03932718901014098</v>
       </c>
       <c r="AY67" t="n">
         <v>-16.71033041805866</v>
@@ -23988,7 +23988,7 @@
         <v>-1.302573977731003</v>
       </c>
       <c r="AY69" t="n">
-        <v>-15.92982162987447</v>
+        <v>-15.92983151621281</v>
       </c>
       <c r="AZ69" t="b">
         <v>0</v>
@@ -24249,7 +24249,7 @@
         <v>1</v>
       </c>
       <c r="V71" t="n">
-        <v>98226323456</v>
+        <v>98502926336</v>
       </c>
       <c r="W71" t="n">
         <v>11.13</v>
@@ -24328,10 +24328,10 @@
         </is>
       </c>
       <c r="AW71" t="n">
-        <v>30.3700008392334</v>
+        <v>30.34000015258789</v>
       </c>
       <c r="AX71" t="n">
-        <v>-7.770828268476048</v>
+        <v>-7.679630560276429</v>
       </c>
       <c r="AY71" t="n">
         <v>-20.69199954808616</v>
@@ -24347,7 +24347,7 @@
       </c>
       <c r="BC71" t="inlineStr">
         <is>
-          <t>sem sinal (-7.8% do topo; Em Baixa)</t>
+          <t>sem sinal (-7.7% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -24495,10 +24495,10 @@
         </is>
       </c>
       <c r="AW72" t="n">
-        <v>4.070000171661377</v>
+        <v>3.990000009536743</v>
       </c>
       <c r="AX72" t="n">
-        <v>-4.422605876297203</v>
+        <v>-2.506263268008835</v>
       </c>
       <c r="AY72" t="n">
         <v>-19.0219927402037</v>
@@ -24514,7 +24514,7 @@
       </c>
       <c r="BC72" t="inlineStr">
         <is>
-          <t>sem sinal (-4.4% do topo; Em Baixa)</t>
+          <t>sem sinal (-2.5% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -24656,10 +24656,10 @@
         </is>
       </c>
       <c r="AW73" t="n">
-        <v>21.27000045776367</v>
+        <v>21.35000038146973</v>
       </c>
       <c r="AX73" t="n">
-        <v>-1.316411286410224</v>
+        <v>-1.686185498450943</v>
       </c>
       <c r="AY73" t="n">
         <v>-23.79046311986899</v>
@@ -24675,7 +24675,7 @@
       </c>
       <c r="BC73" t="inlineStr">
         <is>
-          <t>sem sinal (-1.3% do topo; Em Alta)</t>
+          <t>sem sinal (-1.7% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -25155,7 +25155,7 @@
       <c r="AU76" t="inlineStr"/>
       <c r="AV76" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW76" t="n">
@@ -25178,7 +25178,7 @@
       </c>
       <c r="BC76" t="inlineStr">
         <is>
-          <t>sem sinal (-5.3% do topo; Em Baixa)</t>
+          <t>sem sinal (-5.3% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -25564,7 +25564,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K79" t="n">
@@ -25671,21 +25671,17 @@
       </c>
       <c r="AS79" t="inlineStr"/>
       <c r="AT79" t="inlineStr"/>
-      <c r="AU79" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU79" t="inlineStr"/>
       <c r="AV79" t="inlineStr">
         <is>
           <t>Em Alta</t>
         </is>
       </c>
       <c r="AW79" t="n">
-        <v>3.519999980926514</v>
+        <v>3.559999942779541</v>
       </c>
       <c r="AX79" t="n">
-        <v>0.2840906397000742</v>
+        <v>-0.8426958391001382</v>
       </c>
       <c r="AY79" t="n">
         <v>-43.96825611876666</v>
@@ -25694,14 +25690,14 @@
         <v>0</v>
       </c>
       <c r="BA79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB79" t="b">
         <v>0</v>
       </c>
       <c r="BC79" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (-0.8% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -26085,7 +26081,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K82" t="n">
@@ -26186,21 +26182,17 @@
       </c>
       <c r="AS82" t="inlineStr"/>
       <c r="AT82" t="inlineStr"/>
-      <c r="AU82" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU82" t="inlineStr"/>
       <c r="AV82" t="inlineStr">
         <is>
           <t>Em Baixa</t>
         </is>
       </c>
       <c r="AW82" t="n">
-        <v>21.85000038146973</v>
+        <v>22</v>
       </c>
       <c r="AX82" t="n">
-        <v>0.09153527420819874</v>
+        <v>-0.5909052762118283</v>
       </c>
       <c r="AY82" t="n">
         <v>-14.67030216407054</v>
@@ -26209,14 +26201,14 @@
         <v>0</v>
       </c>
       <c r="BA82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB82" t="b">
         <v>0</v>
       </c>
       <c r="BC82" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (-0.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26350,7 @@
       <c r="AU83" t="inlineStr"/>
       <c r="AV83" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Baixa</t>
         </is>
       </c>
       <c r="AW83" t="n">
@@ -26381,7 +26373,7 @@
       </c>
       <c r="BC83" t="inlineStr">
         <is>
-          <t>sem sinal (-10.4% do topo; Lateral)</t>
+          <t>sem sinal (-10.4% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -26686,10 +26678,10 @@
         </is>
       </c>
       <c r="AW85" t="n">
-        <v>0.1599999964237213</v>
+        <v>0.1700000017881393</v>
       </c>
       <c r="AX85" t="n">
-        <v>0</v>
+        <v>-5.882356034843117</v>
       </c>
       <c r="AY85" t="n">
         <v>-99.17440658744904</v>
@@ -26705,7 +26697,7 @@
       </c>
       <c r="BC85" t="inlineStr">
         <is>
-          <t>sem sinal (+0.0% do topo; Em Baixa)</t>
+          <t>sem sinal (-5.9% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -27867,10 +27859,10 @@
         </is>
       </c>
       <c r="AW92" t="n">
-        <v>66.26999664306641</v>
+        <v>66.09999847412109</v>
       </c>
       <c r="AX92" t="n">
-        <v>-3.561184420100938</v>
+        <v>-3.313159874831761</v>
       </c>
       <c r="AY92" t="n">
         <v>-5.76526078591314</v>
@@ -27886,7 +27878,7 @@
       </c>
       <c r="BC92" t="inlineStr">
         <is>
-          <t>sem sinal (-3.6% do topo; Em Alta)</t>
+          <t>sem sinal (-3.3% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -28376,10 +28368,10 @@
         </is>
       </c>
       <c r="AW95" t="n">
-        <v>21.07999992370605</v>
+        <v>21.17000007629395</v>
       </c>
       <c r="AX95" t="n">
-        <v>-3.889941640379546</v>
+        <v>-4.298534927409481</v>
       </c>
       <c r="AY95" t="n">
         <v>-19.35852192104358</v>
@@ -28395,7 +28387,7 @@
       </c>
       <c r="BC95" t="inlineStr">
         <is>
-          <t>sem sinal (-3.9% do topo; Lateral)</t>
+          <t>sem sinal (-4.3% do topo; Lateral)</t>
         </is>
       </c>
     </row>
@@ -29030,10 +29022,10 @@
         </is>
       </c>
       <c r="AW99" t="n">
-        <v>8.710000038146973</v>
+        <v>8.659999847412109</v>
       </c>
       <c r="AX99" t="n">
-        <v>-0.5740550001823053</v>
+        <v>0</v>
       </c>
       <c r="AY99" t="n">
         <v>-18.43808159694287</v>
@@ -29049,7 +29041,7 @@
       </c>
       <c r="BC99" t="inlineStr">
         <is>
-          <t>sem sinal (-0.6% do topo; Em Baixa)</t>
+          <t>sem sinal (+0.0% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -29372,10 +29364,10 @@
         </is>
       </c>
       <c r="AW101" t="n">
-        <v>32.43999862670898</v>
+        <v>32.27000045776367</v>
       </c>
       <c r="AX101" t="n">
-        <v>-7.12083712617817</v>
+        <v>-6.631550252991147</v>
       </c>
       <c r="AY101" t="n">
         <v>-22.38033148894612</v>
@@ -29391,7 +29383,7 @@
       </c>
       <c r="BC101" t="inlineStr">
         <is>
-          <t>sem sinal (-7.1% do topo; Em Baixa)</t>
+          <t>sem sinal (-6.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -31296,10 +31288,10 @@
         </is>
       </c>
       <c r="AW113" t="n">
-        <v>60.54000091552734</v>
+        <v>60.84999847412109</v>
       </c>
       <c r="AX113" t="n">
-        <v>-3.452263166470892</v>
+        <v>-3.944121234780862</v>
       </c>
       <c r="AY113" t="n">
         <v>-19.90956690277227</v>
@@ -31315,7 +31307,7 @@
       </c>
       <c r="BC113" t="inlineStr">
         <is>
-          <t>sem sinal (-3.5% do topo; Em Alta)</t>
+          <t>sem sinal (-3.9% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -31926,10 +31918,10 @@
         </is>
       </c>
       <c r="AW117" t="n">
-        <v>6.940000057220459</v>
+        <v>6.829999923706055</v>
       </c>
       <c r="AX117" t="n">
-        <v>-15.99423810320502</v>
+        <v>-14.64128859693144</v>
       </c>
       <c r="AY117" t="n">
         <v>-57.6923074261264</v>
@@ -31945,7 +31937,7 @@
       </c>
       <c r="BC117" t="inlineStr">
         <is>
-          <t>sem sinal (-16.0% do topo; Em Baixa)</t>
+          <t>sem sinal (-14.6% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -31985,7 +31977,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="K118" t="n">
@@ -32092,21 +32084,17 @@
       </c>
       <c r="AS118" t="inlineStr"/>
       <c r="AT118" t="inlineStr"/>
-      <c r="AU118" t="inlineStr">
-        <is>
-          <t>Rompimento</t>
-        </is>
-      </c>
+      <c r="AU118" t="inlineStr"/>
       <c r="AV118" t="inlineStr">
         <is>
           <t>Em Alta</t>
         </is>
       </c>
       <c r="AW118" t="n">
-        <v>18.23999977111816</v>
+        <v>18.25</v>
       </c>
       <c r="AX118" t="n">
-        <v>0.05482581692610733</v>
+        <v>0</v>
       </c>
       <c r="AY118" t="n">
         <v>-14.11764705882353</v>
@@ -32115,14 +32103,14 @@
         <v>0</v>
       </c>
       <c r="BA118" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB118" t="b">
         <v>0</v>
       </c>
       <c r="BC118" t="inlineStr">
         <is>
-          <t>Rompimento</t>
+          <t>sem sinal (+0.0% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -32276,10 +32264,10 @@
         </is>
       </c>
       <c r="AW119" t="n">
-        <v>14.27999973297119</v>
+        <v>14.4399995803833</v>
       </c>
       <c r="AX119" t="n">
-        <v>-1.120447131680857</v>
+        <v>-2.21606443298612</v>
       </c>
       <c r="AY119" t="n">
         <v>-18.51651739090506</v>
@@ -32295,7 +32283,7 @@
       </c>
       <c r="BC119" t="inlineStr">
         <is>
-          <t>sem sinal (-1.1% do topo; Em Alta)</t>
+          <t>sem sinal (-2.2% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -33524,10 +33512,10 @@
         </is>
       </c>
       <c r="AW127" t="n">
-        <v>0.3300000131130219</v>
+        <v>0.3100000023841858</v>
       </c>
       <c r="AX127" t="n">
-        <v>-15.15151816185063</v>
+        <v>-9.677419664956521</v>
       </c>
       <c r="AY127" t="n">
         <v>-80.5555562454241</v>
@@ -33543,7 +33531,7 @@
       </c>
       <c r="BC127" t="inlineStr">
         <is>
-          <t>sem sinal (-15.2% do topo; Em Baixa)</t>
+          <t>sem sinal (-9.7% do topo; Em Baixa)</t>
         </is>
       </c>
     </row>
@@ -33689,7 +33677,7 @@
       <c r="AU128" t="inlineStr"/>
       <c r="AV128" t="inlineStr">
         <is>
-          <t>Lateral</t>
+          <t>Em Alta</t>
         </is>
       </c>
       <c r="AW128" t="n">
@@ -33712,7 +33700,7 @@
       </c>
       <c r="BC128" t="inlineStr">
         <is>
-          <t>sem sinal (-1.9% do topo; Lateral)</t>
+          <t>sem sinal (-1.9% do topo; Em Alta)</t>
         </is>
       </c>
     </row>
@@ -34017,10 +34005,10 @@
         </is>
       </c>
       <c r="AW130" t="n">
-        <v>12.31999969482422</v>
+        <v>12.3100004196167</v>
       </c>
       <c r="AX130" t="n">
-        <v>-8.441558341027754</v>
+        <v>-8.367186446266416</v>
       </c>
       <c r="AY130" t="n">
         <v>-23.05593553629934</v>
@@ -34408,7 +34396,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Pivô de alta</t>
         </is>
       </c>
       <c r="K133" t="n">
@@ -34443,7 +34431,7 @@
         <v>0</v>
       </c>
       <c r="V133" t="n">
-        <v>51848818688</v>
+        <v>51957202944</v>
       </c>
       <c r="W133" t="n">
         <v>39.98</v>
@@ -34511,10 +34499,14 @@
       </c>
       <c r="AS133" t="inlineStr"/>
       <c r="AT133" t="inlineStr"/>
-      <c r="AU133" t="inlineStr"/>
+      <c r="AU133" t="inlineStr">
+        <is>
+          <t>Pivô de alta</t>
+        </is>
+      </c>
       <c r="AV133" t="inlineStr">
         <is>
-          <t>Em Baixa</t>
+          <t>Lateral</t>
         </is>
       </c>
       <c r="AW133" t="n">
@@ -34530,14 +34522,14 @@
         <v>0</v>
       </c>
       <c r="BA133" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BB133" t="b">
         <v>0</v>
       </c>
       <c r="BC133" t="inlineStr">
         <is>
-          <t>sem sinal (-0.0% do topo; Em Baixa)</t>
+          <t>Pivô de alta</t>
         </is>
       </c>
     </row>
@@ -34677,7 +34669,7 @@
         <v>-35.41666472641126</v>
       </c>
       <c r="AY134" t="n">
-        <v>-89.31034509690564</v>
+        <v>-89.16083867989796</v>
       </c>
       <c r="AZ134" t="b">
         <v>0</v>

</xml_diff>